<commit_message>
Fix backend startup and test configuration
</commit_message>
<xml_diff>
--- a/backend/scripts/Automated_Answer_Evaluation_Login_Data.xlsx
+++ b/backend/scripts/Automated_Answer_Evaluation_Login_Data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teachers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login_Logs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation_Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Teachers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Admin" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Login_Logs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Evaluation_Results" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4972,6 +4972,288 @@
         </is>
       </c>
       <c r="I101" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>STU101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Demo Student</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>student1784768428@example.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$yt8qDpbV8ro1qSwQ$d4a0baa92ce39e2b0616cb85882d18b0114aca0ff1fb16b2c72610f461c7afaa16f6d1f63db7fb079c26c133fb734d1328df288cbbe2d095b9149a482e4fb142</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>REG0101</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>STU102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>praveen</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>p@gmail.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$6S0BFW0oBX7I7vKY$bbeeb65385fec0646d0bbfeb42cd519e300013fb7d5283455d012733acf540ebddc4cf5459a9a227408487f5d93fc1f96cb887492217b04289e4443f63dd8f7a</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>REG0102</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>STU103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>ututu</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>p123@gmail.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$GvjfiHg8TuYyvr27$e24a5241a5c6a255e1df6cc4c317aa638e2fefdf196df12c322a30469a9eb588130f30914fd9d0c032a889da86fdb2c1dd7b5a9334d0e84020d7d32bb3913384</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>REG0103</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>STU104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>pppprr</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>owjkjfvn@gmail.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$33p164ZPWcVJmAzw$c23a77c5c9d12051f2e87fd8dc91dd3ba2680018ba3fc3e516c723827dcfcc51e5c45213bda32e7b70f538d077df1e4fc612a7f363b32b100d5e83fecc8da353</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>REG0104</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>STU105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>peopewrejopwr</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>owjkjfvndijioh@gmail.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$q4vDftEhHbjXlH1z$082589f22174ab59b15a2510381eec76f0d5b067e8e0257932bb37bd9517b878b0ff8ce6b071457444ba83f9cd0de0e442ed17f0b375ba004a9cafed320bcf76</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>REG0105</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>STU106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$J9wHL9ukAvJrbh3s$712c9cb8a31f52bac59df434fd7a9f89f2da8e468f72e453fde1b517756d0cf9f44cb978ec635331f9556816f5c0ad3105c3e88a7cc08e2c62b9bc6e0ddfa64e</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Not assigned</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>REG0106</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>